<commit_message>
minor tweaks to piano tuning lab
</commit_message>
<xml_diff>
--- a/StudentGuideModule2/piano_tuning/piano_tuning.xlsx
+++ b/StudentGuideModule2/piano_tuning/piano_tuning.xlsx
@@ -1,22 +1,36 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28025"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mtrawick\Desktop\github\132\StudentGuideModule2\piano_tuning\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mtrawick\Box\github\132\StudentGuideModule2\piano_tuning\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B5C3BBE-48D2-4B12-A37F-142BF2260597}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="384" yWindow="36" windowWidth="16260" windowHeight="8736"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="14592" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -81,7 +95,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
@@ -123,27 +137,12 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="4">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -183,19 +182,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="2"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -207,26 +202,27 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -262,7 +258,13 @@
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="4" name="Straight Arrow Connector 3"/>
+        <xdr:cNvPr id="4" name="Straight Arrow Connector 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000004000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
@@ -313,7 +315,13 @@
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="6" name="Straight Connector 5"/>
+        <xdr:cNvPr id="6" name="Straight Connector 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000006000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
@@ -362,7 +370,13 @@
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="9" name="Straight Connector 8"/>
+        <xdr:cNvPr id="9" name="Straight Connector 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000009000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
@@ -411,7 +425,13 @@
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="10" name="Straight Connector 9"/>
+        <xdr:cNvPr id="10" name="Straight Connector 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000A000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
@@ -460,7 +480,13 @@
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="11" name="Straight Arrow Connector 10"/>
+        <xdr:cNvPr id="11" name="Straight Arrow Connector 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000B000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
@@ -511,7 +537,13 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="12" name="TextBox 11"/>
+        <xdr:cNvPr id="12" name="TextBox 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000C000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr txBox="1"/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -577,7 +609,13 @@
       <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
-            <xdr:cNvPr id="13" name="TextBox 12"/>
+            <xdr:cNvPr id="13" name="TextBox 12">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000D000000}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
             <xdr:cNvSpPr txBox="1"/>
           </xdr:nvSpPr>
           <xdr:spPr>
@@ -757,7 +795,13 @@
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="15" name="Straight Arrow Connector 14"/>
+        <xdr:cNvPr id="15" name="Straight Arrow Connector 14">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000F000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvCxnSpPr>
           <a:stCxn id="13" idx="0"/>
         </xdr:cNvCxnSpPr>
@@ -796,13 +840,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>9</xdr:col>
+      <xdr:col>10</xdr:col>
       <xdr:colOff>236220</xdr:colOff>
       <xdr:row>18</xdr:row>
       <xdr:rowOff>144780</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
+      <xdr:col>16</xdr:col>
       <xdr:colOff>365760</xdr:colOff>
       <xdr:row>29</xdr:row>
       <xdr:rowOff>144780</xdr:rowOff>
@@ -811,7 +855,13 @@
       <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
-            <xdr:cNvPr id="17" name="TextBox 16"/>
+            <xdr:cNvPr id="17" name="TextBox 16">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000011000000}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
             <xdr:cNvSpPr txBox="1"/>
           </xdr:nvSpPr>
           <xdr:spPr>
@@ -946,15 +996,18 @@
                     </m:e>
                     <m:sub>
                       <m:r>
-                        <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                        <m:rPr>
+                          <m:sty m:val="p"/>
+                        </m:rPr>
+                        <a:rPr lang="en-US" sz="1100" b="0" i="0">
                           <a:solidFill>
                             <a:sysClr val="windowText" lastClr="000000"/>
                           </a:solidFill>
-                          <a:latin typeface="Cambria Math"/>
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                           <a:ea typeface="+mn-ea"/>
                           <a:cs typeface="+mn-cs"/>
                         </a:rPr>
-                        <m:t>𝐻𝐼𝐺𝐻</m:t>
+                        <m:t>high</m:t>
                       </m:r>
                     </m:sub>
                   </m:sSub>
@@ -1054,15 +1107,18 @@
                     </m:e>
                     <m:sub>
                       <m:r>
-                        <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                        <m:rPr>
+                          <m:sty m:val="p"/>
+                        </m:rPr>
+                        <a:rPr lang="en-US" sz="1100" b="0" i="0">
                           <a:solidFill>
                             <a:sysClr val="windowText" lastClr="000000"/>
                           </a:solidFill>
-                          <a:latin typeface="Cambria Math"/>
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                           <a:ea typeface="+mn-ea"/>
                           <a:cs typeface="+mn-cs"/>
                         </a:rPr>
-                        <m:t>𝐿𝑂𝑊</m:t>
+                        <m:t>low</m:t>
                       </m:r>
                     </m:sub>
                   </m:sSub>
@@ -1167,15 +1223,18 @@
                     </m:e>
                     <m:sub>
                       <m:r>
-                        <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                        <m:rPr>
+                          <m:sty m:val="p"/>
+                        </m:rPr>
+                        <a:rPr lang="en-US" sz="1100" b="0" i="0">
                           <a:solidFill>
                             <a:sysClr val="windowText" lastClr="000000"/>
                           </a:solidFill>
-                          <a:latin typeface="Cambria Math"/>
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                           <a:ea typeface="+mn-ea"/>
                           <a:cs typeface="+mn-cs"/>
                         </a:rPr>
-                        <m:t>𝐿𝑂𝑊</m:t>
+                        <m:t>low</m:t>
                       </m:r>
                     </m:sub>
                   </m:sSub>
@@ -1275,15 +1334,18 @@
                     </m:e>
                     <m:sub>
                       <m:r>
-                        <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                        <m:rPr>
+                          <m:sty m:val="p"/>
+                        </m:rPr>
+                        <a:rPr lang="en-US" sz="1100" b="0" i="0">
                           <a:solidFill>
                             <a:sysClr val="windowText" lastClr="000000"/>
                           </a:solidFill>
-                          <a:latin typeface="Cambria Math"/>
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                           <a:ea typeface="+mn-ea"/>
                           <a:cs typeface="+mn-cs"/>
                         </a:rPr>
-                        <m:t>𝐻𝐼𝐺𝐻</m:t>
+                        <m:t>high</m:t>
                       </m:r>
                     </m:sub>
                   </m:sSub>
@@ -1416,7 +1478,13 @@
       <mc:Fallback>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
-            <xdr:cNvPr id="17" name="TextBox 16"/>
+            <xdr:cNvPr id="17" name="TextBox 16">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000011000000}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
             <xdr:cNvSpPr txBox="1"/>
           </xdr:nvSpPr>
           <xdr:spPr>
@@ -1541,7 +1609,7 @@
                   <a:ea typeface="+mn-ea"/>
                   <a:cs typeface="+mn-cs"/>
                 </a:rPr>
-                <a:t>_</a:t>
+                <a:t>_high</a:t>
               </a:r>
               <a:r>
                 <a:rPr lang="en-US" sz="1100" b="0" i="0">
@@ -1552,7 +1620,7 @@
                   <a:ea typeface="+mn-ea"/>
                   <a:cs typeface="+mn-cs"/>
                 </a:rPr>
-                <a:t>𝐻𝐼𝐺𝐻=</a:t>
+                <a:t>=</a:t>
               </a:r>
               <a:r>
                 <a:rPr lang="en-US" sz="1100" b="0" i="0">
@@ -1629,7 +1697,7 @@
                   <a:ea typeface="+mn-ea"/>
                   <a:cs typeface="+mn-cs"/>
                 </a:rPr>
-                <a:t>_</a:t>
+                <a:t>_low</a:t>
               </a:r>
               <a:r>
                 <a:rPr lang="en-US" sz="1100" b="0" i="0">
@@ -1640,7 +1708,7 @@
                   <a:ea typeface="+mn-ea"/>
                   <a:cs typeface="+mn-cs"/>
                 </a:rPr>
-                <a:t>𝐿𝑂𝑊.</a:t>
+                <a:t>.</a:t>
               </a:r>
               <a:r>
                 <a:rPr lang="en-US" sz="1100" b="0">
@@ -1720,7 +1788,7 @@
                   <a:ea typeface="+mn-ea"/>
                   <a:cs typeface="+mn-cs"/>
                 </a:rPr>
-                <a:t>_</a:t>
+                <a:t>_low</a:t>
               </a:r>
               <a:r>
                 <a:rPr lang="en-US" sz="1100" b="0" i="0">
@@ -1731,7 +1799,7 @@
                   <a:ea typeface="+mn-ea"/>
                   <a:cs typeface="+mn-cs"/>
                 </a:rPr>
-                <a:t>𝐿𝑂𝑊  =</a:t>
+                <a:t>  =</a:t>
               </a:r>
               <a:r>
                 <a:rPr lang="en-US" sz="1100" b="0" i="0">
@@ -1808,18 +1876,7 @@
                   <a:ea typeface="+mn-ea"/>
                   <a:cs typeface="+mn-cs"/>
                 </a:rPr>
-                <a:t>_</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="en-US" sz="1100" b="0" i="0">
-                  <a:solidFill>
-                    <a:sysClr val="windowText" lastClr="000000"/>
-                  </a:solidFill>
-                  <a:latin typeface="Cambria Math"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:rPr>
-                <a:t>𝐻𝐼𝐺𝐻</a:t>
+                <a:t>_high</a:t>
               </a:r>
               <a:r>
                 <a:rPr lang="en-US" sz="1100" b="0">
@@ -1950,22 +2007,28 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>10</xdr:col>
+      <xdr:col>11</xdr:col>
       <xdr:colOff>160020</xdr:colOff>
       <xdr:row>5</xdr:row>
       <xdr:rowOff>45720</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
+      <xdr:col>17</xdr:col>
       <xdr:colOff>99060</xdr:colOff>
       <xdr:row>14</xdr:row>
       <xdr:rowOff>83820</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
-            <xdr:cNvPr id="18" name="TextBox 17"/>
+            <xdr:cNvPr id="18" name="TextBox 17">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000012000000}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
             <xdr:cNvSpPr txBox="1"/>
           </xdr:nvSpPr>
           <xdr:spPr>
@@ -2242,7 +2305,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="18" name="TextBox 17"/>
@@ -2534,7 +2597,13 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="3" name="TextBox 2"/>
+        <xdr:cNvPr id="3" name="TextBox 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000003000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr txBox="1"/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -2599,7 +2668,13 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="14" name="TextBox 13"/>
+        <xdr:cNvPr id="14" name="TextBox 13">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000E000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr txBox="1"/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -2651,22 +2726,28 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
+      <xdr:col>6</xdr:col>
       <xdr:colOff>114300</xdr:colOff>
       <xdr:row>24</xdr:row>
       <xdr:rowOff>30480</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>9</xdr:col>
+      <xdr:col>10</xdr:col>
       <xdr:colOff>30480</xdr:colOff>
       <xdr:row>29</xdr:row>
       <xdr:rowOff>137160</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
-            <xdr:cNvPr id="16" name="TextBox 15"/>
+            <xdr:cNvPr id="16" name="TextBox 15">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000010000000}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
             <xdr:cNvSpPr txBox="1"/>
           </xdr:nvSpPr>
           <xdr:spPr>
@@ -3172,7 +3253,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="16" name="TextBox 15"/>
@@ -3592,20 +3673,26 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
+      <xdr:col>6</xdr:col>
       <xdr:colOff>213360</xdr:colOff>
       <xdr:row>20</xdr:row>
       <xdr:rowOff>68580</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>5</xdr:col>
+      <xdr:col>6</xdr:col>
       <xdr:colOff>449580</xdr:colOff>
       <xdr:row>24</xdr:row>
       <xdr:rowOff>30480</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="2" name="Up Arrow 1"/>
+        <xdr:cNvPr id="2" name="Up Arrow 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -3661,20 +3748,26 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
+      <xdr:col>7</xdr:col>
       <xdr:colOff>255270</xdr:colOff>
       <xdr:row>20</xdr:row>
       <xdr:rowOff>45720</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>9</xdr:col>
+      <xdr:col>10</xdr:col>
       <xdr:colOff>236220</xdr:colOff>
       <xdr:row>22</xdr:row>
       <xdr:rowOff>160020</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="5" name="Bent Arrow 4"/>
+        <xdr:cNvPr id="5" name="Bent Arrow 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000005000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -3731,20 +3824,26 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>8</xdr:col>
+      <xdr:col>9</xdr:col>
       <xdr:colOff>323850</xdr:colOff>
       <xdr:row>14</xdr:row>
       <xdr:rowOff>80010</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
+      <xdr:col>11</xdr:col>
       <xdr:colOff>575310</xdr:colOff>
       <xdr:row>17</xdr:row>
       <xdr:rowOff>72390</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="7" name="U-Turn Arrow 6"/>
+        <xdr:cNvPr id="7" name="U-Turn Arrow 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000007000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -3805,13 +3904,848 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>7620</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>12730</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>122078</xdr:rowOff>
+    </xdr:to>
+    <xdr:grpSp>
+      <xdr:nvGrpSpPr>
+        <xdr:cNvPr id="8" name="Group 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C5D6A595-538D-4EE3-B79B-BF62A925CD23}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGrpSpPr/>
+      </xdr:nvGrpSpPr>
+      <xdr:grpSpPr>
+        <a:xfrm>
+          <a:off x="2636520" y="541020"/>
+          <a:ext cx="1132870" cy="4705508"/>
+          <a:chOff x="2554216" y="530843"/>
+          <a:chExt cx="1103447" cy="4731167"/>
+        </a:xfrm>
+      </xdr:grpSpPr>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="19" name="Straight Connector 18">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EE5C7A76-E1BD-D95A-CAB1-6BC9FFBB7577}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="2554509" y="533774"/>
+            <a:ext cx="0" cy="4725211"/>
+          </a:xfrm>
+          <a:prstGeom prst="line">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:sysClr val="windowText" lastClr="000000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="20" name="Straight Connector 19">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{99900F60-8376-3638-2517-EA5F1E3D85B0}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="2560077" y="855633"/>
+            <a:ext cx="453876" cy="0"/>
+          </a:xfrm>
+          <a:prstGeom prst="line">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:sysClr val="windowText" lastClr="000000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="21" name="Straight Connector 20">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0CF6155E-0958-12B4-0470-18E39687E1B3}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="2560077" y="1170795"/>
+            <a:ext cx="453876" cy="0"/>
+          </a:xfrm>
+          <a:prstGeom prst="line">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:sysClr val="windowText" lastClr="000000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="22" name="Straight Connector 21">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{077F94E1-4F4E-D96A-D04F-FF4178D893FC}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="2560077" y="1485958"/>
+            <a:ext cx="1097586" cy="0"/>
+          </a:xfrm>
+          <a:prstGeom prst="line">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:sysClr val="windowText" lastClr="000000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="23" name="Straight Connector 22">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4044F177-78FE-C300-493F-72E14A4E963C}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="2560077" y="1799624"/>
+            <a:ext cx="453876" cy="0"/>
+          </a:xfrm>
+          <a:prstGeom prst="line">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:sysClr val="windowText" lastClr="000000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="24" name="Straight Connector 23">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C51F8E8E-2E7D-1F16-1F07-A40ECD43DFBB}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="2560077" y="2114786"/>
+            <a:ext cx="453876" cy="0"/>
+          </a:xfrm>
+          <a:prstGeom prst="line">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:sysClr val="windowText" lastClr="000000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="25" name="Straight Connector 24">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F381389C-2E08-A233-497B-992A0C5DC970}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="2560077" y="2429948"/>
+            <a:ext cx="453876" cy="0"/>
+          </a:xfrm>
+          <a:prstGeom prst="line">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:sysClr val="windowText" lastClr="000000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="26" name="Straight Connector 25">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{21D2C19D-C80D-9CFC-BF76-4D63329CCEB3}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="2560077" y="2743615"/>
+            <a:ext cx="1094655" cy="0"/>
+          </a:xfrm>
+          <a:prstGeom prst="line">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:sysClr val="windowText" lastClr="000000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="27" name="Straight Connector 26">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{03C95602-B371-25D9-674D-BCCECA921F3B}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="2560077" y="3058777"/>
+            <a:ext cx="453876" cy="0"/>
+          </a:xfrm>
+          <a:prstGeom prst="line">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:sysClr val="windowText" lastClr="000000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="28" name="Straight Connector 27">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{72016381-B15D-CF4B-343B-B71E428ED8F0}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="2560077" y="3373940"/>
+            <a:ext cx="453876" cy="0"/>
+          </a:xfrm>
+          <a:prstGeom prst="line">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:sysClr val="windowText" lastClr="000000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="29" name="Straight Connector 28">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{59EFDB59-4C2E-4E4F-60A0-C8696BA14F86}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="2560077" y="3689103"/>
+            <a:ext cx="1088794" cy="0"/>
+          </a:xfrm>
+          <a:prstGeom prst="line">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:sysClr val="windowText" lastClr="000000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="30" name="Straight Connector 29">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F407070F-EEDE-E82B-83BE-224C0D43AF62}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="2560077" y="4002769"/>
+            <a:ext cx="453876" cy="0"/>
+          </a:xfrm>
+          <a:prstGeom prst="line">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:sysClr val="windowText" lastClr="000000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="31" name="Straight Connector 30">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4C3219E7-8F80-37FA-CC83-EBB2EE0BDAE5}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="2560077" y="4317931"/>
+            <a:ext cx="453876" cy="0"/>
+          </a:xfrm>
+          <a:prstGeom prst="line">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:sysClr val="windowText" lastClr="000000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="32" name="Straight Connector 31">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8E2AEE97-211E-4F5A-67B8-44EDC3AF45BA}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="2560077" y="4633093"/>
+            <a:ext cx="453876" cy="0"/>
+          </a:xfrm>
+          <a:prstGeom prst="line">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:sysClr val="windowText" lastClr="000000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="33" name="Straight Connector 32">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9DD6D34B-362C-A8A7-836F-C2403D13B4E0}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="2560077" y="4946759"/>
+            <a:ext cx="1081060" cy="0"/>
+          </a:xfrm>
+          <a:prstGeom prst="line">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:sysClr val="windowText" lastClr="000000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="34" name="Straight Connector 33">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2B4773BC-2B3A-A2E9-3F6F-45CF1B8C4530}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="2563008" y="540470"/>
+            <a:ext cx="1085863" cy="0"/>
+          </a:xfrm>
+          <a:prstGeom prst="line">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:sysClr val="windowText" lastClr="000000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="35" name="Straight Connector 34">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F1A6AEB6-5C86-D5CA-7978-A3DDD8DB000F}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="2554216" y="5261916"/>
+            <a:ext cx="467111" cy="0"/>
+          </a:xfrm>
+          <a:prstGeom prst="line">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:sysClr val="windowText" lastClr="000000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="36" name="Straight Connector 35">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7AECDD1D-C4D7-2B38-F007-4BEFCE544BC3}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="3641138" y="530843"/>
+            <a:ext cx="0" cy="4597124"/>
+          </a:xfrm>
+          <a:prstGeom prst="line">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:sysClr val="windowText" lastClr="000000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="37" name="Straight Connector 36">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{924489F0-2C7B-C532-0B80-9954F9C70022}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="3010763" y="5125602"/>
+            <a:ext cx="622623" cy="0"/>
+          </a:xfrm>
+          <a:prstGeom prst="line">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:sysClr val="windowText" lastClr="000000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="38" name="Straight Connector 37">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EEFAA87A-D2CC-898E-0615-31F5E42AA1A6}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="3020571" y="5120877"/>
+            <a:ext cx="0" cy="141133"/>
+          </a:xfrm>
+          <a:prstGeom prst="line">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:sysClr val="windowText" lastClr="000000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+    </xdr:grpSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -3849,9 +4783,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -3886,7 +4820,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -3921,7 +4855,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -4094,242 +5028,257 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I27"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:J29"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="3" max="4" width="8.88671875" customWidth="1"/>
-    <col min="6" max="6" width="8.88671875" style="3"/>
-    <col min="7" max="7" width="11" style="3" customWidth="1"/>
-    <col min="8" max="8" width="8.88671875" style="6"/>
-    <col min="9" max="9" width="14.109375" style="3" customWidth="1"/>
+    <col min="3" max="3" width="8.89453125" customWidth="1"/>
+    <col min="4" max="4" width="9.734375" customWidth="1"/>
+    <col min="5" max="5" width="6.734375" customWidth="1"/>
+    <col min="7" max="7" width="8.89453125" style="1"/>
+    <col min="8" max="8" width="11" style="1" customWidth="1"/>
+    <col min="9" max="9" width="8.89453125" style="4"/>
+    <col min="10" max="10" width="14.1015625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="5">
+    <row r="1" spans="1:10" ht="29.1" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="A1" s="3">
         <f>2^(1/12)</f>
         <v>1.0594630943592953</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="G1" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="G1" s="13" t="s">
+      <c r="H1" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="I1" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="I1" s="7" t="s">
+      <c r="J1" s="5" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="F2" s="8" t="s">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="F2" s="13"/>
+      <c r="G2" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="14" t="s">
+      <c r="H2" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="H2" s="10"/>
-      <c r="I2" s="8" t="s">
+      <c r="I2" s="8"/>
+      <c r="J2" s="6" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="E3" s="1" t="s">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="F3" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="F3" s="3">
+      <c r="G3" s="1">
         <v>130.81278</v>
       </c>
-      <c r="G3" s="15">
+      <c r="H3" s="12">
         <v>130.81278</v>
       </c>
-      <c r="H3" s="11">
+      <c r="I3" s="9">
         <v>1</v>
       </c>
-      <c r="I3" s="3">
+      <c r="J3" s="1">
         <v>130.81278</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="E4" s="2" t="s">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="F4" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="G4" s="15"/>
       <c r="H4" s="12"/>
+      <c r="I4" s="9"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" s="4"/>
-      <c r="E5" s="1" t="s">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="A5" s="2"/>
+      <c r="F5" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="G5" s="15"/>
       <c r="H5" s="12">
+        <f>H10*3/4</f>
+        <v>147.1643775</v>
+      </c>
+      <c r="I5" s="9">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="E6" s="2" t="s">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="F6" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="G6" s="15"/>
       <c r="H6" s="12"/>
+      <c r="I6" s="9"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="E7" s="1" t="s">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="F7" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="G7" s="15"/>
-      <c r="H7" s="12">
+      <c r="H7" s="12"/>
+      <c r="I7" s="9">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="E8" s="1" t="s">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="F8" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="G8" s="15"/>
       <c r="H8" s="12"/>
+      <c r="I8" s="9"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="E9" s="2" t="s">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="F9" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="G9" s="15"/>
-      <c r="H9" s="12">
+      <c r="H9" s="12"/>
+      <c r="I9" s="9">
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="E10" s="1" t="s">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="F10" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="G10" s="15"/>
       <c r="H10" s="12">
+        <f>H3*1.5</f>
+        <v>196.21917000000002</v>
+      </c>
+      <c r="I10" s="9">
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="E11" s="2" t="s">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="F11" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="G11" s="15"/>
-      <c r="H11" s="12">
+      <c r="H11" s="12"/>
+      <c r="I11" s="9">
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="E12" s="1" t="s">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="F12" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="G12" s="15"/>
-      <c r="H12" s="12">
+      <c r="H12" s="12"/>
+      <c r="I12" s="9">
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="E13" s="2" t="s">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="F13" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="G13" s="15"/>
-      <c r="H13" s="12">
+      <c r="H13" s="12"/>
+      <c r="I13" s="9">
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="E14" s="1" t="s">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="F14" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="G14" s="15"/>
-      <c r="H14" s="12">
+      <c r="H14" s="12"/>
+      <c r="I14" s="9">
         <v>6</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="E15" s="1" t="s">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="F15" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="G15" s="15"/>
-      <c r="H15" s="12">
+      <c r="H15" s="12"/>
+      <c r="I15" s="9">
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="E16" s="2" t="s">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="F16" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="G16" s="15"/>
-      <c r="H16" s="12">
+      <c r="H16" s="12"/>
+      <c r="I16" s="9">
         <v>8</v>
       </c>
     </row>
-    <row r="17" spans="5:8" x14ac:dyDescent="0.3">
-      <c r="E17" s="1" t="s">
+    <row r="17" spans="6:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="F17" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="G17" s="15"/>
       <c r="H17" s="12"/>
+      <c r="I17" s="9"/>
     </row>
-    <row r="18" spans="5:8" x14ac:dyDescent="0.3">
-      <c r="E18" s="2" t="s">
+    <row r="18" spans="6:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="F18" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="G18" s="15"/>
-      <c r="H18" s="12">
+      <c r="H18" s="12"/>
+      <c r="I18" s="9">
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="5:8" x14ac:dyDescent="0.3">
-      <c r="E19" s="1" t="s">
+    <row r="19" spans="6:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="F19" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="G19" s="15"/>
       <c r="H19" s="12"/>
+      <c r="I19" s="9"/>
     </row>
-    <row r="20" spans="5:8" x14ac:dyDescent="0.3">
-      <c r="E20" s="1" t="s">
+    <row r="20" spans="6:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="F20" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="G20" s="15"/>
-      <c r="H20" s="12">
+      <c r="H20" s="12"/>
+      <c r="I20" s="9">
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="5:8" x14ac:dyDescent="0.3">
-      <c r="E21" s="2" t="s">
+    <row r="21" spans="6:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="F21" s="14" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="22" spans="5:8" x14ac:dyDescent="0.3">
-      <c r="E22" s="1" t="s">
+    <row r="22" spans="6:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="F22" s="13" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="23" spans="5:8" x14ac:dyDescent="0.3">
-      <c r="E23" s="2" t="s">
+    <row r="23" spans="6:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="F23" s="14" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="24" spans="5:8" x14ac:dyDescent="0.3">
-      <c r="E24" s="1" t="s">
+    <row r="24" spans="6:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="F24" s="13" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="25" spans="5:8" x14ac:dyDescent="0.3">
-      <c r="E25" s="2" t="s">
+    <row r="25" spans="6:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="F25" s="14" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="26" spans="5:8" x14ac:dyDescent="0.3">
-      <c r="E26" s="1" t="s">
+    <row r="26" spans="6:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="F26" s="13" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="27" spans="5:8" x14ac:dyDescent="0.3">
-      <c r="E27" s="1" t="s">
+    <row r="27" spans="6:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="F27" s="13" t="s">
         <v>0</v>
       </c>
+    </row>
+    <row r="28" spans="6:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="F28" s="13"/>
+    </row>
+    <row r="29" spans="6:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="F29" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4338,18 +5287,18 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>